<commit_message>
chore: translate updated scenarios
</commit_message>
<xml_diff>
--- a/魔物娘TD_名字编号属性对照表.xlsx
+++ b/魔物娘TD_名字编号属性对照表.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9853" uniqueCount="2469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2531" uniqueCount="2531">
   <si>
     <t>编号</t>
   </si>
@@ -7443,6 +7443,192 @@
   </si>
   <si>
     <t>编号、稀有度、种族名、日文名、属性、初期职业、武器、类型、攻击类型、配置类型、移动类型及基础属性</t>
+  </si>
+  <si>
+    <t>469</t>
+  </si>
+  <si>
+    <t>バエル娘</t>
+  </si>
+  <si>
+    <t>15 / 魔法剣</t>
+  </si>
+  <si>
+    <t>悪魔/進化</t>
+  </si>
+  <si>
+    <t>2166</t>
+  </si>
+  <si>
+    <t>468</t>
+  </si>
+  <si>
+    <t>フェネクス娘</t>
+  </si>
+  <si>
+    <t>43 / ブーメラン</t>
+  </si>
+  <si>
+    <t>1764</t>
+  </si>
+  <si>
+    <t>467</t>
+  </si>
+  <si>
+    <t>ライトニンググリフォン娘</t>
+  </si>
+  <si>
+    <t>魔獣/進化</t>
+  </si>
+  <si>
+    <t>1506</t>
+  </si>
+  <si>
+    <t>ベルグリシ娘</t>
+  </si>
+  <si>
+    <t>デミ/進化</t>
+  </si>
+  <si>
+    <t>4485</t>
+  </si>
+  <si>
+    <t>夜戯のアラクネ娘</t>
+  </si>
+  <si>
+    <t>1508</t>
+  </si>
+  <si>
+    <t>魔戯猫グリマルキン娘</t>
+  </si>
+  <si>
+    <t>魔獣</t>
+  </si>
+  <si>
+    <t>2185</t>
+  </si>
+  <si>
+    <t>463</t>
+  </si>
+  <si>
+    <t>戯触のローパー娘</t>
+  </si>
+  <si>
+    <t>462</t>
+  </si>
+  <si>
+    <t>ハッグ娘</t>
+  </si>
+  <si>
+    <t>ドルゼフィーダ</t>
+  </si>
+  <si>
+    <t>461</t>
+  </si>
+  <si>
+    <t>ティアマト娘</t>
+  </si>
+  <si>
+    <t>ティアマリア</t>
+  </si>
+  <si>
+    <t>ドラゴン/海魔/禁忌</t>
+  </si>
+  <si>
+    <t>2356</t>
+  </si>
+  <si>
+    <t>598</t>
+  </si>
+  <si>
+    <t>プロメテウス娘</t>
+  </si>
+  <si>
+    <t>メテリナ</t>
+  </si>
+  <si>
+    <t>デミ/禁忌</t>
+  </si>
+  <si>
+    <t>459</t>
+  </si>
+  <si>
+    <t>フェンリル娘</t>
+  </si>
+  <si>
+    <t>エリル</t>
+  </si>
+  <si>
+    <t>魔獣/禁忌</t>
+  </si>
+  <si>
+    <t>禁忌の神殿</t>
+  </si>
+  <si>
+    <t>458</t>
+  </si>
+  <si>
+    <t>ワーキャット娘</t>
+  </si>
+  <si>
+    <t>ミャルナ</t>
+  </si>
+  <si>
+    <t>デミ/魔獣</t>
+  </si>
+  <si>
+    <t>457</t>
+  </si>
+  <si>
+    <t>T.O.W.E.R.typeM</t>
+  </si>
+  <si>
+    <t>ティヴェル</t>
+  </si>
+  <si>
+    <t>456</t>
+  </si>
+  <si>
+    <t>コズミックモーフ娘</t>
+  </si>
+  <si>
+    <t>ヴォミラ</t>
+  </si>
+  <si>
+    <t>1490</t>
+  </si>
+  <si>
+    <t>フライング・ヒューマノイド娘</t>
+  </si>
+  <si>
+    <t>シエルナ</t>
+  </si>
+  <si>
+    <t>454</t>
+  </si>
+  <si>
+    <t>ヴィーナシアン娘</t>
+  </si>
+  <si>
+    <t>ルキーナ</t>
+  </si>
+  <si>
+    <t>3905</t>
+  </si>
+  <si>
+    <t>453</t>
+  </si>
+  <si>
+    <t>ケルピー娘</t>
+  </si>
+  <si>
+    <t>ストリオーネ</t>
+  </si>
+  <si>
+    <t>1107</t>
+  </si>
+  <si>
+    <t>進化</t>
   </si>
 </sst>
 </file>
@@ -8335,7 +8521,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:V453"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
@@ -8551,6 +8737,9 @@
       <c r="V3" t="s">
         <v>42</v>
       </c>
+      <c r="J3" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="4" spans="1:22">
       <c r="A4" t="s">
@@ -8752,6 +8941,9 @@
       <c r="V6" t="s">
         <v>42</v>
       </c>
+      <c r="J6" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="7" spans="1:22">
       <c r="A7" t="s">
@@ -9157,6 +9349,9 @@
       <c r="V12" t="s">
         <v>42</v>
       </c>
+      <c r="J12" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="13" spans="1:22">
       <c r="A13" t="s">
@@ -9494,6 +9689,9 @@
       <c r="V17" t="s">
         <v>42</v>
       </c>
+      <c r="J17" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="18" spans="1:22">
       <c r="A18" t="s">
@@ -9757,6 +9955,9 @@
       <c r="V21" t="s">
         <v>42</v>
       </c>
+      <c r="J21" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="22" spans="1:22">
       <c r="A22" t="s">
@@ -9890,6 +10091,9 @@
       <c r="V23" t="s">
         <v>42</v>
       </c>
+      <c r="J23" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="24" spans="1:22">
       <c r="A24" t="s">
@@ -10620,6 +10824,9 @@
       <c r="V34" t="s">
         <v>42</v>
       </c>
+      <c r="J34" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="35" spans="1:22">
       <c r="A35" t="s">
@@ -11084,6 +11291,9 @@
       <c r="V41" t="s">
         <v>42</v>
       </c>
+      <c r="J41" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="42" spans="1:22">
       <c r="A42" t="s">
@@ -11616,6 +11826,9 @@
       <c r="V49" t="s">
         <v>494</v>
       </c>
+      <c r="J49" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="50" spans="1:22">
       <c r="A50" t="s">
@@ -11749,6 +11962,9 @@
       <c r="V51" t="s">
         <v>494</v>
       </c>
+      <c r="J51" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="52" spans="1:22">
       <c r="A52" t="s">
@@ -11879,6 +12095,9 @@
       <c r="V53" t="s">
         <v>42</v>
       </c>
+      <c r="J53" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="54" spans="1:22">
       <c r="A54" t="s">
@@ -12012,6 +12231,9 @@
       <c r="V55" t="s">
         <v>42</v>
       </c>
+      <c r="J55" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="56" spans="1:22">
       <c r="A56" t="s">
@@ -12275,6 +12497,9 @@
       <c r="V59" t="s">
         <v>42</v>
       </c>
+      <c r="J59" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="60" spans="1:22">
       <c r="A60" t="s">
@@ -12538,6 +12763,9 @@
       <c r="V63" t="s">
         <v>42</v>
       </c>
+      <c r="J63" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="64" spans="1:22">
       <c r="A64" t="s">
@@ -12603,6 +12831,9 @@
       <c r="V64" t="s">
         <v>42</v>
       </c>
+      <c r="J64" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="65" spans="1:22">
       <c r="A65" t="s">
@@ -12804,6 +13035,9 @@
       <c r="V67" t="s">
         <v>42</v>
       </c>
+      <c r="J67" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68" t="s">
@@ -12869,6 +13103,9 @@
       <c r="V68" t="s">
         <v>494</v>
       </c>
+      <c r="J68" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="69" spans="1:22">
       <c r="A69" t="s">
@@ -13002,6 +13239,9 @@
       <c r="V70" t="s">
         <v>42</v>
       </c>
+      <c r="J70" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="71" spans="1:22">
       <c r="A71" t="s">
@@ -13868,6 +14108,9 @@
       <c r="V83" t="s">
         <v>42</v>
       </c>
+      <c r="J83" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="84" spans="1:22">
       <c r="A84" t="s">
@@ -14069,6 +14312,9 @@
       <c r="V86" t="s">
         <v>42</v>
       </c>
+      <c r="J86" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="87" spans="1:22">
       <c r="A87" t="s">
@@ -14134,6 +14380,9 @@
       <c r="V87" t="s">
         <v>42</v>
       </c>
+      <c r="J87" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="88" spans="1:22">
       <c r="A88" t="s">
@@ -14403,6 +14652,9 @@
       <c r="V91" t="s">
         <v>42</v>
       </c>
+      <c r="J91" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="92" spans="1:22">
       <c r="A92" t="s">
@@ -14604,6 +14856,9 @@
       <c r="V94" t="s">
         <v>42</v>
       </c>
+      <c r="J94" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="95" spans="1:22">
       <c r="A95" t="s">
@@ -15331,6 +15586,9 @@
       <c r="V105" t="s">
         <v>494</v>
       </c>
+      <c r="J105" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="106" spans="1:22">
       <c r="A106" t="s">
@@ -16132,6 +16390,9 @@
       <c r="V117" t="s">
         <v>494</v>
       </c>
+      <c r="J117" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="118" spans="1:22">
       <c r="A118" t="s">
@@ -17409,6 +17670,9 @@
       <c r="V136" t="s">
         <v>1041</v>
       </c>
+      <c r="J136" t="s">
+        <v>2480</v>
+      </c>
     </row>
     <row r="137" spans="1:22">
       <c r="A137" t="s">
@@ -20658,6 +20922,9 @@
       <c r="V184" t="s">
         <v>494</v>
       </c>
+      <c r="J184" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="185" spans="1:22">
       <c r="A185" t="s">
@@ -20791,6 +21058,9 @@
       <c r="V186" t="s">
         <v>1041</v>
       </c>
+      <c r="J186" t="s">
+        <v>2530</v>
+      </c>
     </row>
     <row r="187" spans="1:22">
       <c r="A187" t="s">
@@ -21193,6 +21463,9 @@
       <c r="V192" t="s">
         <v>494</v>
       </c>
+      <c r="J192" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="193" spans="1:22">
       <c r="A193" t="s">
@@ -21326,6 +21599,9 @@
       <c r="V194" t="s">
         <v>42</v>
       </c>
+      <c r="J194" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="195" spans="1:22">
       <c r="A195" t="s">
@@ -22003,6 +22279,9 @@
       <c r="V204" t="s">
         <v>42</v>
       </c>
+      <c r="J204" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="205" spans="1:22">
       <c r="A205" t="s">
@@ -23954,6 +24233,9 @@
       <c r="V233" t="s">
         <v>42</v>
       </c>
+      <c r="J233" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="234" spans="1:22">
       <c r="A234" t="s">
@@ -24291,6 +24573,9 @@
       <c r="V238" t="s">
         <v>966</v>
       </c>
+      <c r="J238" t="s">
+        <v>2530</v>
+      </c>
     </row>
     <row r="239" spans="1:22">
       <c r="A239" t="s">
@@ -24560,6 +24845,9 @@
       <c r="V242" t="s">
         <v>494</v>
       </c>
+      <c r="J242" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="243" spans="1:22">
       <c r="A243" t="s">
@@ -26452,6 +26740,9 @@
       <c r="V270" t="s">
         <v>42</v>
       </c>
+      <c r="J270" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="271" spans="1:22">
       <c r="A271" t="s">
@@ -27401,6 +27692,9 @@
       <c r="V284" t="s">
         <v>1041</v>
       </c>
+      <c r="J284" t="s">
+        <v>2530</v>
+      </c>
     </row>
     <row r="285" spans="1:22">
       <c r="A285" t="s">
@@ -27466,6 +27760,9 @@
       <c r="V285" t="s">
         <v>1041</v>
       </c>
+      <c r="J285" t="s">
+        <v>2530</v>
+      </c>
     </row>
     <row r="286" spans="1:22">
       <c r="A286" t="s">
@@ -28551,6 +28848,9 @@
       <c r="V301" t="s">
         <v>42</v>
       </c>
+      <c r="J301" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="302" spans="1:22">
       <c r="A302" t="s">
@@ -30295,6 +30595,9 @@
       <c r="V327" t="s">
         <v>494</v>
       </c>
+      <c r="J327" t="s">
+        <v>2530</v>
+      </c>
     </row>
     <row r="328" spans="1:22">
       <c r="A328" t="s">
@@ -30972,6 +31275,9 @@
       <c r="V337" t="s">
         <v>42</v>
       </c>
+      <c r="J337" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="338" spans="1:22">
       <c r="A338" t="s">
@@ -32258,6 +32564,9 @@
       <c r="V356" t="s">
         <v>494</v>
       </c>
+      <c r="J356" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="357" spans="1:22">
       <c r="A357" t="s">
@@ -34691,6 +35000,9 @@
       <c r="V392" t="s">
         <v>42</v>
       </c>
+      <c r="J392" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="393" spans="1:22">
       <c r="A393" t="s">
@@ -35025,6 +35337,9 @@
       <c r="V397" t="s">
         <v>1553</v>
       </c>
+      <c r="J397" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="398" spans="1:22">
       <c r="A398" t="s">
@@ -35220,6 +35535,9 @@
       <c r="V400" t="s">
         <v>966</v>
       </c>
+      <c r="J400" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="401" spans="1:22">
       <c r="A401" t="s">
@@ -35622,6 +35940,9 @@
       <c r="V406" t="s">
         <v>42</v>
       </c>
+      <c r="J406" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="407" spans="1:22">
       <c r="A407" t="s">
@@ -35956,6 +36277,9 @@
       <c r="V411" t="s">
         <v>42</v>
       </c>
+      <c r="J411" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="412" spans="1:22">
       <c r="A412" t="s">
@@ -36157,6 +36481,9 @@
       <c r="V414" t="s">
         <v>555</v>
       </c>
+      <c r="J414" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="415" spans="1:22">
       <c r="A415" t="s">
@@ -36494,6 +36821,9 @@
       <c r="V419" t="s">
         <v>555</v>
       </c>
+      <c r="J419" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="420" spans="1:22">
       <c r="A420" t="s">
@@ -36695,6 +37025,9 @@
       <c r="V422" t="s">
         <v>966</v>
       </c>
+      <c r="J422" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="423" spans="1:22">
       <c r="A423" t="s">
@@ -36964,6 +37297,9 @@
       <c r="V426" t="s">
         <v>966</v>
       </c>
+      <c r="J426" t="s">
+        <v>2530</v>
+      </c>
     </row>
     <row r="427" ht="19.5" customHeight="1" spans="1:22">
       <c r="A427" t="s">
@@ -38043,6 +38379,9 @@
       <c r="V442" t="s">
         <v>42</v>
       </c>
+      <c r="J442" t="s">
+        <v>2488</v>
+      </c>
     </row>
     <row r="443" spans="1:22">
       <c r="A443" t="s">
@@ -38786,8 +39125,1056 @@
         <v>966</v>
       </c>
     </row>
+    <row r="454" spans="1:22">
+      <c r="A454" t="s">
+        <v>2469</v>
+      </c>
+      <c r="B454" t="s">
+        <v>23</v>
+      </c>
+      <c r="C454" t="s">
+        <v>2470</v>
+      </c>
+      <c r="D454" t="s">
+        <v>1468</v>
+      </c>
+      <c r="G454" t="s">
+        <v>166</v>
+      </c>
+      <c r="H454" t="s">
+        <v>48</v>
+      </c>
+      <c r="I454" t="s">
+        <v>2471</v>
+      </c>
+      <c r="J454" t="s">
+        <v>2472</v>
+      </c>
+      <c r="K454" t="s">
+        <v>207</v>
+      </c>
+      <c r="L454" t="s">
+        <v>51</v>
+      </c>
+      <c r="M454" t="s">
+        <v>52</v>
+      </c>
+      <c r="N454" t="s">
+        <v>2473</v>
+      </c>
+      <c r="O454" t="s">
+        <v>723</v>
+      </c>
+      <c r="P454" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q454" t="s">
+        <v>854</v>
+      </c>
+      <c r="R454" t="s">
+        <v>57</v>
+      </c>
+      <c r="S454" t="s">
+        <v>313</v>
+      </c>
+      <c r="T454" t="s">
+        <v>58</v>
+      </c>
+      <c r="U454" t="s">
+        <v>41</v>
+      </c>
+      <c r="V454" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="455" spans="1:22">
+      <c r="A455" t="s">
+        <v>2474</v>
+      </c>
+      <c r="B455" t="s">
+        <v>23</v>
+      </c>
+      <c r="C455" t="s">
+        <v>2475</v>
+      </c>
+      <c r="D455" t="s">
+        <v>25</v>
+      </c>
+      <c r="G455" t="s">
+        <v>28</v>
+      </c>
+      <c r="H455" t="s">
+        <v>205</v>
+      </c>
+      <c r="I455" t="s">
+        <v>2476</v>
+      </c>
+      <c r="J455" t="s">
+        <v>2472</v>
+      </c>
+      <c r="K455" t="s">
+        <v>50</v>
+      </c>
+      <c r="L455" t="s">
+        <v>32</v>
+      </c>
+      <c r="M455" t="s">
+        <v>33</v>
+      </c>
+      <c r="N455" t="s">
+        <v>2477</v>
+      </c>
+      <c r="O455" t="s">
+        <v>1540</v>
+      </c>
+      <c r="P455" t="s">
+        <v>979</v>
+      </c>
+      <c r="Q455" t="s">
+        <v>221</v>
+      </c>
+      <c r="R455" t="s">
+        <v>38</v>
+      </c>
+      <c r="S455" t="s">
+        <v>965</v>
+      </c>
+      <c r="T455" t="s">
+        <v>58</v>
+      </c>
+      <c r="U455" t="s">
+        <v>73</v>
+      </c>
+      <c r="V455" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="456" spans="1:22">
+      <c r="A456" t="s">
+        <v>2478</v>
+      </c>
+      <c r="B456" t="s">
+        <v>23</v>
+      </c>
+      <c r="C456" t="s">
+        <v>2479</v>
+      </c>
+      <c r="D456" t="s">
+        <v>532</v>
+      </c>
+      <c r="G456" t="s">
+        <v>157</v>
+      </c>
+      <c r="H456" t="s">
+        <v>205</v>
+      </c>
+      <c r="I456" t="s">
+        <v>217</v>
+      </c>
+      <c r="J456" t="s">
+        <v>2480</v>
+      </c>
+      <c r="K456" t="s">
+        <v>50</v>
+      </c>
+      <c r="L456" t="s">
+        <v>32</v>
+      </c>
+      <c r="M456" t="s">
+        <v>33</v>
+      </c>
+      <c r="N456" t="s">
+        <v>2481</v>
+      </c>
+      <c r="O456" t="s">
+        <v>871</v>
+      </c>
+      <c r="P456" t="s">
+        <v>909</v>
+      </c>
+      <c r="Q456" t="s">
+        <v>56</v>
+      </c>
+      <c r="R456" t="s">
+        <v>38</v>
+      </c>
+      <c r="S456" t="s">
+        <v>257</v>
+      </c>
+      <c r="T456" t="s">
+        <v>72</v>
+      </c>
+      <c r="U456" t="s">
+        <v>85</v>
+      </c>
+      <c r="V456" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="457" spans="1:22">
+      <c r="A457" t="s">
+        <v>954</v>
+      </c>
+      <c r="B457" t="s">
+        <v>23</v>
+      </c>
+      <c r="C457" t="s">
+        <v>2482</v>
+      </c>
+      <c r="D457" t="s">
+        <v>497</v>
+      </c>
+      <c r="G457" t="s">
+        <v>157</v>
+      </c>
+      <c r="H457" t="s">
+        <v>48</v>
+      </c>
+      <c r="I457" t="s">
+        <v>49</v>
+      </c>
+      <c r="J457" t="s">
+        <v>2483</v>
+      </c>
+      <c r="K457" t="s">
+        <v>50</v>
+      </c>
+      <c r="L457" t="s">
+        <v>51</v>
+      </c>
+      <c r="M457" t="s">
+        <v>436</v>
+      </c>
+      <c r="N457" t="s">
+        <v>2484</v>
+      </c>
+      <c r="O457" t="s">
+        <v>1871</v>
+      </c>
+      <c r="P457" t="s">
+        <v>1222</v>
+      </c>
+      <c r="Q457" t="s">
+        <v>56</v>
+      </c>
+      <c r="R457" t="s">
+        <v>140</v>
+      </c>
+      <c r="S457" t="s">
+        <v>38</v>
+      </c>
+      <c r="T457" t="s">
+        <v>58</v>
+      </c>
+      <c r="U457" t="s">
+        <v>350</v>
+      </c>
+      <c r="V457" t="s">
+        <v>1553</v>
+      </c>
+    </row>
+    <row r="458" spans="1:22">
+      <c r="A458" t="s">
+        <v>2078</v>
+      </c>
+      <c r="B458" t="s">
+        <v>23</v>
+      </c>
+      <c r="C458" t="s">
+        <v>2485</v>
+      </c>
+      <c r="D458" t="s">
+        <v>512</v>
+      </c>
+      <c r="G458" t="s">
+        <v>92</v>
+      </c>
+      <c r="H458" t="s">
+        <v>205</v>
+      </c>
+      <c r="I458" t="s">
+        <v>217</v>
+      </c>
+      <c r="K458" t="s">
+        <v>50</v>
+      </c>
+      <c r="L458" t="s">
+        <v>32</v>
+      </c>
+      <c r="M458" t="s">
+        <v>436</v>
+      </c>
+      <c r="N458" t="s">
+        <v>2486</v>
+      </c>
+      <c r="O458" t="s">
+        <v>82</v>
+      </c>
+      <c r="P458" t="s">
+        <v>909</v>
+      </c>
+      <c r="Q458" t="s">
+        <v>283</v>
+      </c>
+      <c r="R458" t="s">
+        <v>211</v>
+      </c>
+      <c r="S458" t="s">
+        <v>257</v>
+      </c>
+      <c r="T458" t="s">
+        <v>72</v>
+      </c>
+      <c r="U458" t="s">
+        <v>85</v>
+      </c>
+      <c r="V458" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="459" spans="1:22">
+      <c r="A459" t="s">
+        <v>501</v>
+      </c>
+      <c r="B459" t="s">
+        <v>23</v>
+      </c>
+      <c r="C459" t="s">
+        <v>2487</v>
+      </c>
+      <c r="D459" t="s">
+        <v>2228</v>
+      </c>
+      <c r="G459" t="s">
+        <v>28</v>
+      </c>
+      <c r="H459" t="s">
+        <v>48</v>
+      </c>
+      <c r="I459" t="s">
+        <v>2471</v>
+      </c>
+      <c r="J459" t="s">
+        <v>2488</v>
+      </c>
+      <c r="K459" t="s">
+        <v>207</v>
+      </c>
+      <c r="L459" t="s">
+        <v>51</v>
+      </c>
+      <c r="M459" t="s">
+        <v>52</v>
+      </c>
+      <c r="N459" t="s">
+        <v>2489</v>
+      </c>
+      <c r="O459" t="s">
+        <v>2116</v>
+      </c>
+      <c r="P459" t="s">
+        <v>972</v>
+      </c>
+      <c r="Q459" t="s">
+        <v>854</v>
+      </c>
+      <c r="R459" t="s">
+        <v>57</v>
+      </c>
+      <c r="S459" t="s">
+        <v>313</v>
+      </c>
+      <c r="T459" t="s">
+        <v>58</v>
+      </c>
+      <c r="U459" t="s">
+        <v>41</v>
+      </c>
+      <c r="V459" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="460" spans="1:22">
+      <c r="A460" t="s">
+        <v>2490</v>
+      </c>
+      <c r="B460" t="s">
+        <v>75</v>
+      </c>
+      <c r="C460" t="s">
+        <v>2491</v>
+      </c>
+      <c r="D460" t="s">
+        <v>443</v>
+      </c>
+      <c r="G460" t="s">
+        <v>65</v>
+      </c>
+      <c r="H460" t="s">
+        <v>289</v>
+      </c>
+      <c r="I460" t="s">
+        <v>290</v>
+      </c>
+      <c r="J460" t="s">
+        <v>187</v>
+      </c>
+      <c r="K460" t="s">
+        <v>207</v>
+      </c>
+      <c r="L460" t="s">
+        <v>32</v>
+      </c>
+      <c r="M460" t="s">
+        <v>52</v>
+      </c>
+      <c r="N460" t="s">
+        <v>2404</v>
+      </c>
+      <c r="O460" t="s">
+        <v>2159</v>
+      </c>
+      <c r="P460" t="s">
+        <v>348</v>
+      </c>
+      <c r="Q460" t="s">
+        <v>902</v>
+      </c>
+      <c r="R460" t="s">
+        <v>211</v>
+      </c>
+      <c r="S460" t="s">
+        <v>294</v>
+      </c>
+      <c r="T460" t="s">
+        <v>180</v>
+      </c>
+      <c r="U460" t="s">
+        <v>117</v>
+      </c>
+      <c r="V460" t="s">
+        <v>1553</v>
+      </c>
+    </row>
+    <row r="461" spans="1:22">
+      <c r="A461" t="s">
+        <v>2492</v>
+      </c>
+      <c r="B461" t="s">
+        <v>23</v>
+      </c>
+      <c r="C461" t="s">
+        <v>2493</v>
+      </c>
+      <c r="D461" t="s">
+        <v>2494</v>
+      </c>
+      <c r="G461" t="s">
+        <v>166</v>
+      </c>
+      <c r="H461" t="s">
+        <v>289</v>
+      </c>
+      <c r="I461" t="s">
+        <v>1697</v>
+      </c>
+      <c r="K461" t="s">
+        <v>207</v>
+      </c>
+      <c r="L461" t="s">
+        <v>427</v>
+      </c>
+      <c r="M461" t="s">
+        <v>52</v>
+      </c>
+      <c r="N461" t="s">
+        <v>1743</v>
+      </c>
+      <c r="O461" t="s">
+        <v>871</v>
+      </c>
+      <c r="P461" t="s">
+        <v>301</v>
+      </c>
+      <c r="Q461" t="s">
+        <v>1229</v>
+      </c>
+      <c r="R461" t="s">
+        <v>38</v>
+      </c>
+      <c r="S461" t="s">
+        <v>294</v>
+      </c>
+      <c r="T461" t="s">
+        <v>40</v>
+      </c>
+      <c r="U461" t="s">
+        <v>314</v>
+      </c>
+      <c r="V461" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="462" spans="1:22">
+      <c r="A462" t="s">
+        <v>2495</v>
+      </c>
+      <c r="B462" t="s">
+        <v>23</v>
+      </c>
+      <c r="C462" t="s">
+        <v>2496</v>
+      </c>
+      <c r="D462" t="s">
+        <v>2497</v>
+      </c>
+      <c r="G462" t="s">
+        <v>65</v>
+      </c>
+      <c r="H462" t="s">
+        <v>48</v>
+      </c>
+      <c r="I462" t="s">
+        <v>2471</v>
+      </c>
+      <c r="J462" t="s">
+        <v>2498</v>
+      </c>
+      <c r="K462" t="s">
+        <v>207</v>
+      </c>
+      <c r="L462" t="s">
+        <v>51</v>
+      </c>
+      <c r="M462" t="s">
+        <v>33</v>
+      </c>
+      <c r="N462" t="s">
+        <v>2499</v>
+      </c>
+      <c r="O462" t="s">
+        <v>2500</v>
+      </c>
+      <c r="P462" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q462" t="s">
+        <v>1147</v>
+      </c>
+      <c r="R462" t="s">
+        <v>57</v>
+      </c>
+      <c r="S462" t="s">
+        <v>69</v>
+      </c>
+      <c r="T462" t="s">
+        <v>58</v>
+      </c>
+      <c r="U462" t="s">
+        <v>96</v>
+      </c>
+      <c r="V462" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="463" spans="1:22">
+      <c r="A463" t="s">
+        <v>1136</v>
+      </c>
+      <c r="B463" t="s">
+        <v>23</v>
+      </c>
+      <c r="C463" t="s">
+        <v>2501</v>
+      </c>
+      <c r="D463" t="s">
+        <v>2502</v>
+      </c>
+      <c r="G463" t="s">
+        <v>28</v>
+      </c>
+      <c r="H463" t="s">
+        <v>29</v>
+      </c>
+      <c r="I463" t="s">
+        <v>365</v>
+      </c>
+      <c r="J463" t="s">
+        <v>2503</v>
+      </c>
+      <c r="K463" t="s">
+        <v>31</v>
+      </c>
+      <c r="L463" t="s">
+        <v>32</v>
+      </c>
+      <c r="M463" t="s">
+        <v>52</v>
+      </c>
+      <c r="N463" t="s">
+        <v>1186</v>
+      </c>
+      <c r="O463" t="s">
+        <v>1504</v>
+      </c>
+      <c r="P463" t="s">
+        <v>538</v>
+      </c>
+      <c r="Q463" t="s">
+        <v>916</v>
+      </c>
+      <c r="R463" t="s">
+        <v>211</v>
+      </c>
+      <c r="S463" t="s">
+        <v>522</v>
+      </c>
+      <c r="T463" t="s">
+        <v>370</v>
+      </c>
+      <c r="U463" t="s">
+        <v>348</v>
+      </c>
+      <c r="V463" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="464" spans="1:22">
+      <c r="A464" t="s">
+        <v>2504</v>
+      </c>
+      <c r="B464" t="s">
+        <v>23</v>
+      </c>
+      <c r="C464" t="s">
+        <v>2505</v>
+      </c>
+      <c r="D464" t="s">
+        <v>2506</v>
+      </c>
+      <c r="G464" t="s">
+        <v>92</v>
+      </c>
+      <c r="H464" t="s">
+        <v>205</v>
+      </c>
+      <c r="I464" t="s">
+        <v>2476</v>
+      </c>
+      <c r="J464" t="s">
+        <v>2507</v>
+      </c>
+      <c r="K464" t="s">
+        <v>50</v>
+      </c>
+      <c r="L464" t="s">
+        <v>32</v>
+      </c>
+      <c r="M464" t="s">
+        <v>52</v>
+      </c>
+      <c r="N464" t="s">
+        <v>774</v>
+      </c>
+      <c r="O464" t="s">
+        <v>1907</v>
+      </c>
+      <c r="P464" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q464" t="s">
+        <v>128</v>
+      </c>
+      <c r="R464" t="s">
+        <v>211</v>
+      </c>
+      <c r="S464" t="s">
+        <v>965</v>
+      </c>
+      <c r="T464" t="s">
+        <v>58</v>
+      </c>
+      <c r="U464" t="s">
+        <v>84</v>
+      </c>
+      <c r="V464" t="s">
+        <v>2508</v>
+      </c>
+    </row>
+    <row r="465" spans="1:22">
+      <c r="A465" t="s">
+        <v>2509</v>
+      </c>
+      <c r="B465" t="s">
+        <v>75</v>
+      </c>
+      <c r="C465" t="s">
+        <v>2510</v>
+      </c>
+      <c r="D465" t="s">
+        <v>2511</v>
+      </c>
+      <c r="G465" t="s">
+        <v>186</v>
+      </c>
+      <c r="H465" t="s">
+        <v>289</v>
+      </c>
+      <c r="I465" t="s">
+        <v>1697</v>
+      </c>
+      <c r="J465" t="s">
+        <v>2512</v>
+      </c>
+      <c r="K465" t="s">
+        <v>207</v>
+      </c>
+      <c r="L465" t="s">
+        <v>32</v>
+      </c>
+      <c r="M465" t="s">
+        <v>52</v>
+      </c>
+      <c r="N465" t="s">
+        <v>1796</v>
+      </c>
+      <c r="O465" t="s">
+        <v>150</v>
+      </c>
+      <c r="P465" t="s">
+        <v>264</v>
+      </c>
+      <c r="Q465" t="s">
+        <v>1187</v>
+      </c>
+      <c r="R465" t="s">
+        <v>211</v>
+      </c>
+      <c r="S465" t="s">
+        <v>39</v>
+      </c>
+      <c r="T465" t="s">
+        <v>40</v>
+      </c>
+      <c r="U465" t="s">
+        <v>41</v>
+      </c>
+      <c r="V465" t="s">
+        <v>1553</v>
+      </c>
+    </row>
+    <row r="466" spans="1:22">
+      <c r="A466" t="s">
+        <v>2513</v>
+      </c>
+      <c r="B466" t="s">
+        <v>23</v>
+      </c>
+      <c r="C466" t="s">
+        <v>2514</v>
+      </c>
+      <c r="D466" t="s">
+        <v>2515</v>
+      </c>
+      <c r="G466" t="s">
+        <v>166</v>
+      </c>
+      <c r="H466" t="s">
+        <v>48</v>
+      </c>
+      <c r="I466" t="s">
+        <v>66</v>
+      </c>
+      <c r="J466" t="s">
+        <v>885</v>
+      </c>
+      <c r="K466" t="s">
+        <v>50</v>
+      </c>
+      <c r="L466" t="s">
+        <v>51</v>
+      </c>
+      <c r="M466" t="s">
+        <v>52</v>
+      </c>
+      <c r="N466" t="s">
+        <v>826</v>
+      </c>
+      <c r="O466" t="s">
+        <v>1766</v>
+      </c>
+      <c r="P466" t="s">
+        <v>627</v>
+      </c>
+      <c r="Q466" t="s">
+        <v>554</v>
+      </c>
+      <c r="R466" t="s">
+        <v>57</v>
+      </c>
+      <c r="S466" t="s">
+        <v>58</v>
+      </c>
+      <c r="T466" t="s">
+        <v>72</v>
+      </c>
+      <c r="U466" t="s">
+        <v>73</v>
+      </c>
+      <c r="V466" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="467" spans="1:22">
+      <c r="A467" t="s">
+        <v>2516</v>
+      </c>
+      <c r="B467" t="s">
+        <v>23</v>
+      </c>
+      <c r="C467" t="s">
+        <v>2517</v>
+      </c>
+      <c r="D467" t="s">
+        <v>2518</v>
+      </c>
+      <c r="G467" t="s">
+        <v>166</v>
+      </c>
+      <c r="H467" t="s">
+        <v>425</v>
+      </c>
+      <c r="I467" t="s">
+        <v>1167</v>
+      </c>
+      <c r="J467" t="s">
+        <v>1577</v>
+      </c>
+      <c r="K467" t="s">
+        <v>50</v>
+      </c>
+      <c r="L467" t="s">
+        <v>427</v>
+      </c>
+      <c r="M467" t="s">
+        <v>52</v>
+      </c>
+      <c r="N467" t="s">
+        <v>2519</v>
+      </c>
+      <c r="O467" t="s">
+        <v>1345</v>
+      </c>
+      <c r="P467" t="s">
+        <v>523</v>
+      </c>
+      <c r="Q467" t="s">
+        <v>1089</v>
+      </c>
+      <c r="R467" t="s">
+        <v>211</v>
+      </c>
+      <c r="S467" t="s">
+        <v>1170</v>
+      </c>
+      <c r="T467" t="s">
+        <v>563</v>
+      </c>
+      <c r="U467" t="s">
+        <v>85</v>
+      </c>
+      <c r="V467" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="468" spans="1:22">
+      <c r="A468" t="s">
+        <v>1528</v>
+      </c>
+      <c r="B468" t="s">
+        <v>23</v>
+      </c>
+      <c r="C468" t="s">
+        <v>2520</v>
+      </c>
+      <c r="D468" t="s">
+        <v>2521</v>
+      </c>
+      <c r="G468" t="s">
+        <v>166</v>
+      </c>
+      <c r="H468" t="s">
+        <v>425</v>
+      </c>
+      <c r="I468" t="s">
+        <v>535</v>
+      </c>
+      <c r="J468" t="s">
+        <v>1577</v>
+      </c>
+      <c r="K468" t="s">
+        <v>50</v>
+      </c>
+      <c r="L468" t="s">
+        <v>427</v>
+      </c>
+      <c r="M468" t="s">
+        <v>33</v>
+      </c>
+      <c r="N468" t="s">
+        <v>1560</v>
+      </c>
+      <c r="O468" t="s">
+        <v>688</v>
+      </c>
+      <c r="P468" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q468" t="s">
+        <v>171</v>
+      </c>
+      <c r="R468" t="s">
+        <v>38</v>
+      </c>
+      <c r="S468" t="s">
+        <v>430</v>
+      </c>
+      <c r="T468" t="s">
+        <v>58</v>
+      </c>
+      <c r="U468" t="s">
+        <v>73</v>
+      </c>
+      <c r="V468" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="469" spans="1:22">
+      <c r="A469" t="s">
+        <v>2522</v>
+      </c>
+      <c r="B469" t="s">
+        <v>23</v>
+      </c>
+      <c r="C469" t="s">
+        <v>2523</v>
+      </c>
+      <c r="D469" t="s">
+        <v>2524</v>
+      </c>
+      <c r="G469" t="s">
+        <v>92</v>
+      </c>
+      <c r="H469" t="s">
+        <v>134</v>
+      </c>
+      <c r="I469" t="s">
+        <v>147</v>
+      </c>
+      <c r="J469" t="s">
+        <v>1577</v>
+      </c>
+      <c r="K469" t="s">
+        <v>50</v>
+      </c>
+      <c r="L469" t="s">
+        <v>51</v>
+      </c>
+      <c r="M469" t="s">
+        <v>52</v>
+      </c>
+      <c r="N469" t="s">
+        <v>2525</v>
+      </c>
+      <c r="O469" t="s">
+        <v>188</v>
+      </c>
+      <c r="P469" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q469" t="s">
+        <v>151</v>
+      </c>
+      <c r="R469" t="s">
+        <v>140</v>
+      </c>
+      <c r="S469" t="s">
+        <v>38</v>
+      </c>
+      <c r="T469" t="s">
+        <v>40</v>
+      </c>
+      <c r="U469" t="s">
+        <v>554</v>
+      </c>
+      <c r="V469" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="470" spans="1:22">
+      <c r="A470" t="s">
+        <v>2526</v>
+      </c>
+      <c r="B470" t="s">
+        <v>23</v>
+      </c>
+      <c r="C470" t="s">
+        <v>2527</v>
+      </c>
+      <c r="D470" t="s">
+        <v>2528</v>
+      </c>
+      <c r="G470" t="s">
+        <v>65</v>
+      </c>
+      <c r="H470" t="s">
+        <v>289</v>
+      </c>
+      <c r="I470" t="s">
+        <v>1697</v>
+      </c>
+      <c r="J470" t="s">
+        <v>401</v>
+      </c>
+      <c r="K470" t="s">
+        <v>207</v>
+      </c>
+      <c r="L470" t="s">
+        <v>427</v>
+      </c>
+      <c r="M470" t="s">
+        <v>52</v>
+      </c>
+      <c r="N470" t="s">
+        <v>2529</v>
+      </c>
+      <c r="O470" t="s">
+        <v>1766</v>
+      </c>
+      <c r="P470" t="s">
+        <v>840</v>
+      </c>
+      <c r="Q470" t="s">
+        <v>127</v>
+      </c>
+      <c r="R470" t="s">
+        <v>211</v>
+      </c>
+      <c r="S470" t="s">
+        <v>294</v>
+      </c>
+      <c r="T470" t="s">
+        <v>40</v>
+      </c>
+      <c r="U470" t="s">
+        <v>314</v>
+      </c>
+      <c r="V470" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:V453" etc:filterBottomFollowUsedRange="0">
+  <autoFilter ref="A1:V453" ns1:filterBottomFollowUsedRange="0">
     <sortState ref="A1:V453">
       <sortCondition ref="A1:A453"/>
     </sortState>

</xml_diff>